<commit_message>
Atualiza ficha admissional: e-mail, escolaridade, estado civil e CNH
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CZYfs53cnUXnhZ6z1qeekx
</commit_message>
<xml_diff>
--- a/ficha_maria/FICHA_ADMISSIONAL_MARIA_EDUARDA.xlsx
+++ b/ficha_maria/FICHA_ADMISSIONAL_MARIA_EDUARDA.xlsx
@@ -834,14 +834,19 @@
           <t>Telefone fixo</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>NÃO TEM</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>FALTA</t>
+          <t>Mensagem do usuário</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Preenchido</t>
         </is>
       </c>
     </row>
@@ -883,14 +888,19 @@
           <t>E-mail</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>eduardadandrade18@gmail.com</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>FALTA</t>
+          <t>Mensagem do usuário</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Preenchido</t>
         </is>
       </c>
     </row>
@@ -986,14 +996,19 @@
           <t>Grau de instrução</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Ensino médio completo (2º Grau completo)</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>FALTA (CNIS em branco)</t>
+          <t>Mensagem do usuário</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Preenchido</t>
         </is>
       </c>
     </row>
@@ -1008,14 +1023,19 @@
           <t>Curso / Data conclusão</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>NÃO TEM</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>FALTA</t>
+          <t>Mensagem do usuário</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Preenchido</t>
         </is>
       </c>
     </row>
@@ -1030,14 +1050,19 @@
           <t>Estado civil / Casamento / Cônjuge</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>SOLTEIRA</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>FALTA</t>
+          <t>Mensagem do usuário</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Preenchido</t>
         </is>
       </c>
     </row>
@@ -1285,14 +1310,19 @@
           <t>Habilitação (CNH)</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>EM ANDAMENTO</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>FALTA / não possui?</t>
+          <t>Mensagem do usuário</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Preenchido</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza ficha admissional: raça/cor, reservista, dependentes e VT
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CZYfs53cnUXnhZ6z1qeekx
</commit_message>
<xml_diff>
--- a/ficha_maria/FICHA_ADMISSIONAL_MARIA_EDUARDA.xlsx
+++ b/ficha_maria/FICHA_ADMISSIONAL_MARIA_EDUARDA.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1077,14 +1077,19 @@
           <t>Raça/Cor</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BRANCA</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>FALTA</t>
+          <t>Mensagem do usuário</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Preenchido</t>
         </is>
       </c>
     </row>
@@ -1418,14 +1423,19 @@
           <t>Reservista</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>NÃO TEM</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>FALTA</t>
+          <t>Mensagem do usuário</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Preenchido</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1555,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Estrangeiro / Dependentes / Benefícios (exceto VT)</t>
+          <t>Estrangeiro / % desconto VT / outros benefícios</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1599,7 +1609,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Sim (valor diário não informado)</t>
+          <t>Sim – valor diário R$ 12,00 (% desconto não informado)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1689,6 +1699,33 @@
         </is>
       </c>
       <c r="E47" t="inlineStr">
+        <is>
+          <t>Preenchido</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Dependentes</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Dependentes (IR / salário família)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>NÃO TEM</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Mensagem do usuário</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>Preenchido</t>
         </is>

</xml_diff>

<commit_message>
Atualiza ficha admissional: deficiência (nenhuma) e desconto do VT (6%)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CZYfs53cnUXnhZ6z1qeekx
</commit_message>
<xml_diff>
--- a/ficha_maria/FICHA_ADMISSIONAL_MARIA_EDUARDA.xlsx
+++ b/ficha_maria/FICHA_ADMISSIONAL_MARIA_EDUARDA.xlsx
@@ -1104,14 +1104,19 @@
           <t>Deficiente</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>NENHUMA</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>FALTA</t>
+          <t>Mensagem do usuário</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Preenchido</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1560,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Estrangeiro / % desconto VT / outros benefícios</t>
+          <t>Estrangeiro / outros benefícios</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1609,7 +1614,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Sim – valor diário R$ 12,00 (% desconto não informado)</t>
+          <t>Sim – R$ 12,00/dia – 6% de desconto</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">

</xml_diff>

<commit_message>
Ficha admissional: confirma nome da médica do ASO
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CZYfs53cnUXnhZ6z1qeekx
</commit_message>
<xml_diff>
--- a/ficha_maria/FICHA_ADMISSIONAL_MARIA_EDUARDA.xlsx
+++ b/ficha_maria/FICHA_ADMISSIONAL_MARIA_EDUARDA.xlsx
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Dra. Ana Carolina de Sena Lem… (sobrenome cortado)</t>
+          <t>Dra. Ana Carolina de Sena Lem…</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1519,9 +1519,9 @@
           <t>ASO</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>CONFERIR sobrenome completo</t>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Confirmado pelo usuário</t>
         </is>
       </c>
     </row>

</xml_diff>